<commit_message>
Modify sample input to TACC employees
</commit_message>
<xml_diff>
--- a/example_input.xlsx
+++ b/example_input.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10402"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kbeavers/Documents/GitHub/publication-scraper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2A30A5E-5464-824A-822F-5D4CD0989011}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D671AB66-9D67-C043-A9F3-DB89CB04D27B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2280" yWindow="980" windowWidth="27640" windowHeight="16940" xr2:uid="{D894F065-5AA2-3F42-93CB-4D37D05B9DC2}"/>
   </bookViews>
   <sheets>
     <sheet name="utrc_active_allocations" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
   <si>
     <t>root_institution_name</t>
   </si>
@@ -60,15 +60,6 @@
   </si>
   <si>
     <t>James</t>
-  </si>
-  <si>
-    <t>Mydlarz</t>
-  </si>
-  <si>
-    <t>Laura</t>
-  </si>
-  <si>
-    <t>The University of Texas at Arlington</t>
   </si>
 </sst>
 </file>
@@ -495,15 +486,9 @@
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>